<commit_message>
Updated  issues to include bug in planned keep-in zone approach.
</commit_message>
<xml_diff>
--- a/doc/assurance/ZoneAlertService/4-Issues/issues.xlsx
+++ b/doc/assurance/ZoneAlertService/4-Issues/issues.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10714"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10916"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Dependable/Contracts/ASTRA/Deliverables/OpenUxAS-ZoneAlert/doc/assurance/ZoneAlertService/5-Issues/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Dependable/Contracts/ASTRA/Deliverables/OpenUxAS-ZoneAlert/doc/assurance/ZoneAlertService/4-Issues/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD86FC0C-F7CA-C64F-B813-B97440806F83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20861C20-4B6C-7B48-9F09-CF084A4FC409}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="200" yWindow="500" windowWidth="33760" windowHeight="20740" xr2:uid="{C9A58872-7F3C-C947-8C7B-D579EDD417B1}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="75">
   <si>
     <t>Status</t>
   </si>
@@ -254,6 +254,15 @@
   </si>
   <si>
     <t>Process argument eliminated from problem argument in favor of direct reasoning</t>
+  </si>
+  <si>
+    <t>Solution exploration revealed that our code has the wrong model of keep-in zone semantics. Should store the first keep-in zone that each is in if any. If  in one at start, violation occurs if leave all overlapping keep-ins including starting one. Otherwise if not in one, then no keep-in zone violation will occur.</t>
+  </si>
+  <si>
+    <t>Continue to work on problem diagram and its temporal form, reach conclusion state</t>
+  </si>
+  <si>
+    <t>Maintain both classical problem frames diagram as well as solution exploration diagram</t>
   </si>
 </sst>
 </file>
@@ -694,7 +703,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50891FDD-30FA-7E4F-8B50-3438F693C3DF}">
-  <dimension ref="A1:I48"/>
+  <dimension ref="A1:I51"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.5" style="10" customWidth="1"/>
@@ -1461,6 +1470,42 @@
       </c>
       <c r="I48" t="s">
         <v>8</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="G49" s="4">
+        <v>45566</v>
+      </c>
+      <c r="H49" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="I49" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="G50" s="4">
+        <v>45589</v>
+      </c>
+      <c r="H50" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="I50" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" ht="102" x14ac:dyDescent="0.2">
+      <c r="A51" s="10">
+        <v>13</v>
+      </c>
+      <c r="B51" t="s">
+        <v>8</v>
+      </c>
+      <c r="C51" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="E51" s="4">
+        <v>45595</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated issue list to reflect current project state.
</commit_message>
<xml_diff>
--- a/doc/assurance/ZoneAlertService/4-Issues/issues.xlsx
+++ b/doc/assurance/ZoneAlertService/4-Issues/issues.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Dependable/Contracts/ASTRA/Deliverables/OpenUxAS-ZoneAlert/doc/assurance/ZoneAlertService/4-Issues/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20861C20-4B6C-7B48-9F09-CF084A4FC409}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1FCC447-AE31-4A41-9284-7272EB4EF17F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="200" yWindow="500" windowWidth="33760" windowHeight="20740" xr2:uid="{C9A58872-7F3C-C947-8C7B-D579EDD417B1}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="85">
   <si>
     <t>Status</t>
   </si>
@@ -262,7 +262,37 @@
     <t>Continue to work on problem diagram and its temporal form, reach conclusion state</t>
   </si>
   <si>
+    <t>CLOSED</t>
+  </si>
+  <si>
     <t>Maintain both classical problem frames diagram as well as solution exploration diagram</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>Updated documents to reflect keep-in zone behavior</t>
+  </si>
+  <si>
+    <t>Continued work to update documentation for vehicle behavior and solution specificaiton</t>
+  </si>
+  <si>
+    <t>Noted an alternative solution that only considers last keep-in zone the vehicel is in on its last state report.</t>
+  </si>
+  <si>
+    <t>Discussed options for solution with stakeholders</t>
+  </si>
+  <si>
+    <t>Updated documentation and graphs to show selected behavior and solution approach</t>
+  </si>
+  <si>
+    <t>Having developed problem frame and soltion exploration diagram formats as part of research, this question is resolved to our satisfaction.</t>
+  </si>
+  <si>
+    <t>Decided to code a copy of zone merge that is tech debt</t>
+  </si>
+  <si>
+    <t>Tech Debt: Zone Merge Code is a copy of semantics obseved elsewhere. Result duplicate zone merging computation with slightly different semantics in various OpenUxAS Services.</t>
   </si>
 </sst>
 </file>
@@ -703,7 +733,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50891FDD-30FA-7E4F-8B50-3438F693C3DF}">
-  <dimension ref="A1:I51"/>
+  <dimension ref="A1:I57"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.5" style="10" customWidth="1"/>
@@ -1042,7 +1072,7 @@
         <v>1.2</v>
       </c>
       <c r="B21" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="C21" s="6" t="s">
         <v>26</v>
@@ -1050,6 +1080,9 @@
       <c r="E21" s="4">
         <v>45320</v>
       </c>
+      <c r="F21" s="9">
+        <v>45444</v>
+      </c>
       <c r="G21" s="4">
         <v>45321</v>
       </c>
@@ -1060,198 +1093,201 @@
         <v>8</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="68" x14ac:dyDescent="0.2">
-      <c r="A22" s="10">
+    <row r="22" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="G22" s="4">
+        <v>45444</v>
+      </c>
+      <c r="H22" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="I22" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="68" x14ac:dyDescent="0.2">
+      <c r="A23" s="10">
         <v>5</v>
       </c>
-      <c r="B22" t="s">
-        <v>20</v>
-      </c>
-      <c r="C22" s="6" t="s">
+      <c r="B23" t="s">
+        <v>20</v>
+      </c>
+      <c r="C23" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="E22" s="4">
+      <c r="E23" s="4">
         <v>45320</v>
       </c>
-      <c r="F22" s="9">
+      <c r="F23" s="9">
         <v>45320</v>
       </c>
-      <c r="G22" s="4">
-        <v>45320</v>
-      </c>
-      <c r="H22" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="I22" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" ht="85" x14ac:dyDescent="0.2">
       <c r="G23" s="4">
         <v>45320</v>
       </c>
       <c r="H23" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="I23" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="85" x14ac:dyDescent="0.2">
+      <c r="G24" s="4">
+        <v>45320</v>
+      </c>
+      <c r="H24" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="I23" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A24" s="10">
+      <c r="I24" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="A25" s="10">
         <v>1.3</v>
       </c>
-      <c r="B24" t="s">
-        <v>20</v>
-      </c>
-      <c r="C24" s="6" t="s">
+      <c r="B25" t="s">
+        <v>20</v>
+      </c>
+      <c r="C25" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="E24" s="4">
-        <v>45321</v>
-      </c>
-      <c r="F24" s="9">
-        <v>45321</v>
-      </c>
-      <c r="G24" s="4">
-        <v>45321</v>
-      </c>
-      <c r="H24" s="6" t="s">
+      <c r="E25" s="4">
+        <v>45321</v>
+      </c>
+      <c r="F25" s="9">
+        <v>45321</v>
+      </c>
+      <c r="G25" s="4">
+        <v>45321</v>
+      </c>
+      <c r="H25" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="I24" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" ht="51" x14ac:dyDescent="0.2">
-      <c r="A25" s="10">
+      <c r="I25" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" ht="51" x14ac:dyDescent="0.2">
+      <c r="A26" s="10">
         <v>1.4</v>
       </c>
-      <c r="B25" t="s">
-        <v>20</v>
-      </c>
-      <c r="C25" s="6" t="s">
+      <c r="B26" t="s">
+        <v>20</v>
+      </c>
+      <c r="C26" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="E25" s="4">
-        <v>45321</v>
-      </c>
-      <c r="G25" s="4">
+      <c r="E26" s="4">
+        <v>45321</v>
+      </c>
+      <c r="F26" s="9">
+        <v>45312</v>
+      </c>
+      <c r="G26" s="4">
         <v>45322</v>
       </c>
-      <c r="H25" s="6" t="s">
+      <c r="H26" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="I25" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" ht="187" x14ac:dyDescent="0.2">
-      <c r="A26" s="10">
+      <c r="I26" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" ht="187" x14ac:dyDescent="0.2">
+      <c r="A27" s="10">
         <v>6</v>
       </c>
-      <c r="B26" t="s">
-        <v>20</v>
-      </c>
-      <c r="C26" s="6" t="s">
+      <c r="B27" t="s">
+        <v>20</v>
+      </c>
+      <c r="C27" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="E26" s="4">
-        <v>45321</v>
-      </c>
-      <c r="F26" s="9">
-        <v>45321</v>
-      </c>
-      <c r="G26" s="4">
-        <v>45321</v>
-      </c>
-      <c r="H26" s="6" t="s">
+      <c r="E27" s="4">
+        <v>45321</v>
+      </c>
+      <c r="F27" s="9">
+        <v>45321</v>
+      </c>
+      <c r="G27" s="4">
+        <v>45321</v>
+      </c>
+      <c r="H27" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="I26" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9" ht="68" x14ac:dyDescent="0.2">
-      <c r="A27" s="10">
+      <c r="I27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" ht="68" x14ac:dyDescent="0.2">
+      <c r="A28" s="10">
         <v>7</v>
       </c>
-      <c r="B27" t="s">
-        <v>20</v>
-      </c>
-      <c r="C27" s="6" t="s">
+      <c r="B28" t="s">
+        <v>20</v>
+      </c>
+      <c r="C28" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="E27" s="4">
-        <v>45321</v>
-      </c>
-      <c r="F27" s="9">
-        <v>45321</v>
-      </c>
-      <c r="G27" s="4">
-        <v>45321</v>
-      </c>
-      <c r="H27" s="6" t="s">
+      <c r="E28" s="4">
+        <v>45321</v>
+      </c>
+      <c r="F28" s="9">
+        <v>45321</v>
+      </c>
+      <c r="G28" s="4">
+        <v>45321</v>
+      </c>
+      <c r="H28" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="I27" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9" ht="119" x14ac:dyDescent="0.2">
-      <c r="A28" s="10">
-        <v>8</v>
-      </c>
-      <c r="B28" t="s">
-        <v>20</v>
-      </c>
-      <c r="C28" s="6" t="s">
+      <c r="I28" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" ht="119" x14ac:dyDescent="0.2">
+      <c r="A29" s="10">
+        <v>8</v>
+      </c>
+      <c r="B29" t="s">
+        <v>20</v>
+      </c>
+      <c r="C29" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="E28" s="4">
-        <v>45321</v>
-      </c>
-      <c r="F28" s="9">
-        <v>45321</v>
-      </c>
-      <c r="G28" s="4">
-        <v>45321</v>
-      </c>
-      <c r="H28" s="6" t="s">
+      <c r="E29" s="4">
+        <v>45321</v>
+      </c>
+      <c r="F29" s="9">
+        <v>45321</v>
+      </c>
+      <c r="G29" s="4">
+        <v>45321</v>
+      </c>
+      <c r="H29" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="I28" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9" ht="51" x14ac:dyDescent="0.2">
-      <c r="G29" s="4">
-        <v>45321</v>
-      </c>
-      <c r="H29" s="6" t="s">
+      <c r="I29" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" ht="51" x14ac:dyDescent="0.2">
+      <c r="G30" s="4">
+        <v>45321</v>
+      </c>
+      <c r="H30" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="I29" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="G30" s="4">
-        <v>45321</v>
-      </c>
-      <c r="H30" s="6" t="s">
+      <c r="I30" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="G31" s="4">
+        <v>45321</v>
+      </c>
+      <c r="H31" s="6" t="s">
         <v>44</v>
-      </c>
-      <c r="I30" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="G31" s="4">
-        <v>45321</v>
-      </c>
-      <c r="H31" s="6" t="s">
-        <v>45</v>
       </c>
       <c r="I31" t="s">
         <v>8</v>
@@ -1262,112 +1298,121 @@
         <v>45321</v>
       </c>
       <c r="H32" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="I32" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="G33" s="4">
+        <v>45321</v>
+      </c>
+      <c r="H33" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="I32" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A33" s="10">
+      <c r="I33" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="A34" s="10">
         <v>9</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B34" t="s">
         <v>68</v>
       </c>
-      <c r="C33" s="6" t="s">
+      <c r="C34" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="E33" s="4">
-        <v>45321</v>
-      </c>
-      <c r="F33" s="9">
+      <c r="E34" s="4">
+        <v>45321</v>
+      </c>
+      <c r="F34" s="9">
         <v>45352</v>
       </c>
-      <c r="G33" s="4">
+      <c r="G34" s="4">
         <v>45352</v>
       </c>
-      <c r="H33" s="6" t="s">
+      <c r="H34" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="I33" t="s">
+      <c r="I34" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="34" spans="1:9" ht="68" x14ac:dyDescent="0.2">
-      <c r="A34" s="10">
+    <row r="35" spans="1:9" ht="68" x14ac:dyDescent="0.2">
+      <c r="A35" s="10">
         <v>10</v>
       </c>
-      <c r="B34" t="s">
-        <v>8</v>
-      </c>
-      <c r="C34" s="6" t="s">
+      <c r="B35" t="s">
+        <v>74</v>
+      </c>
+      <c r="C35" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="E34" s="4">
-        <v>45321</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A35" s="10">
+      <c r="E35" s="4">
+        <v>45321</v>
+      </c>
+      <c r="G35" s="4">
+        <v>45607</v>
+      </c>
+      <c r="H35" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="I35" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="A36" s="10">
         <v>11</v>
       </c>
-      <c r="B35" t="s">
-        <v>20</v>
-      </c>
-      <c r="C35" s="6" t="s">
+      <c r="B36" t="s">
+        <v>20</v>
+      </c>
+      <c r="C36" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="E35" s="4">
-        <v>45321</v>
-      </c>
-      <c r="F35" s="9">
+      <c r="E36" s="4">
+        <v>45321</v>
+      </c>
+      <c r="F36" s="9">
         <v>45494</v>
       </c>
-      <c r="I35" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="G36" s="4">
+      <c r="I36" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="G37" s="4">
         <v>45494</v>
       </c>
-      <c r="H36" s="6" t="s">
+      <c r="H37" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="I36" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" ht="68" x14ac:dyDescent="0.2">
-      <c r="A37" s="10">
+      <c r="I37" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" ht="68" x14ac:dyDescent="0.2">
+      <c r="A38" s="10">
         <v>12</v>
       </c>
-      <c r="B37" t="s">
-        <v>8</v>
-      </c>
-      <c r="C37" s="6" t="s">
+      <c r="B38" t="s">
+        <v>8</v>
+      </c>
+      <c r="C38" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="E37" s="4">
+      <c r="E38" s="4">
         <v>45379</v>
       </c>
-      <c r="G37" s="4">
+      <c r="G38" s="4">
         <v>45379</v>
       </c>
-      <c r="H37" s="6" t="s">
+      <c r="H38" s="6" t="s">
         <v>57</v>
-      </c>
-      <c r="I37" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="G38" s="4">
-        <v>45446</v>
-      </c>
-      <c r="H38" s="6" t="s">
-        <v>58</v>
       </c>
       <c r="I38" t="s">
         <v>8</v>
@@ -1375,87 +1420,90 @@
     </row>
     <row r="39" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="G39" s="4">
-        <v>45447</v>
+        <v>45446</v>
       </c>
       <c r="H39" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="I39" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="40" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="G40" s="4">
         <v>45447</v>
       </c>
       <c r="H40" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="I40" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="A41" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="G41" s="4">
+        <v>45447</v>
+      </c>
+      <c r="H41" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="I40" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="G42" s="4">
+      <c r="I41" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="G43" s="4">
         <v>45447</v>
       </c>
-      <c r="H42" s="6" t="s">
+      <c r="H43" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="I42" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="G43" s="4">
-        <v>45478</v>
-      </c>
-      <c r="H43" s="6" t="s">
-        <v>64</v>
-      </c>
       <c r="I43" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="44" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="G44" s="4">
         <v>45478</v>
       </c>
       <c r="H44" s="6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I44" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="45" spans="1:9" ht="51" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="G45" s="4">
         <v>45478</v>
       </c>
       <c r="H45" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="I45" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" ht="51" x14ac:dyDescent="0.2">
+      <c r="G46" s="4">
+        <v>45478</v>
+      </c>
+      <c r="H46" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="I45" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="46" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="G46" s="4">
+      <c r="I46" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="G47" s="4">
         <v>45482</v>
       </c>
-      <c r="H46" s="6" t="s">
+      <c r="H47" s="6" t="s">
         <v>67</v>
-      </c>
-      <c r="I46" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="G47" s="4">
-        <v>45483</v>
-      </c>
-      <c r="H47" s="6" t="s">
-        <v>69</v>
       </c>
       <c r="I47" t="s">
         <v>8</v>
@@ -1463,10 +1511,10 @@
     </row>
     <row r="48" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="G48" s="4">
-        <v>45494</v>
+        <v>45483</v>
       </c>
       <c r="H48" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="I48" t="s">
         <v>8</v>
@@ -1474,10 +1522,10 @@
     </row>
     <row r="49" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="G49" s="4">
-        <v>45566</v>
+        <v>45494</v>
       </c>
       <c r="H49" s="6" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="I49" t="s">
         <v>8</v>
@@ -1485,27 +1533,108 @@
     </row>
     <row r="50" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="G50" s="4">
+        <v>45566</v>
+      </c>
+      <c r="H50" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="I50" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="G51" s="4">
         <v>45589</v>
       </c>
-      <c r="H50" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="I50" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="51" spans="1:9" ht="102" x14ac:dyDescent="0.2">
-      <c r="A51" s="10">
+      <c r="H51" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="I51" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" ht="102" x14ac:dyDescent="0.2">
+      <c r="A52" s="10">
         <v>13</v>
       </c>
-      <c r="B51" t="s">
-        <v>8</v>
-      </c>
-      <c r="C51" s="6" t="s">
+      <c r="B52" t="s">
+        <v>20</v>
+      </c>
+      <c r="C52" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="E51" s="4">
+      <c r="E52" s="4">
         <v>45595</v>
+      </c>
+      <c r="F52" s="9">
+        <v>45607</v>
+      </c>
+      <c r="G52" s="4">
+        <v>45595</v>
+      </c>
+      <c r="H52" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="I52" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="G53" s="4">
+        <v>45600</v>
+      </c>
+      <c r="H53" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="I53" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="G54" s="4">
+        <v>45607</v>
+      </c>
+      <c r="H54" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="I54" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="G55" s="4">
+        <v>45607</v>
+      </c>
+      <c r="H55" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="I55" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="G56" s="4">
+        <v>45607</v>
+      </c>
+      <c r="H56" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="I56" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" ht="68" x14ac:dyDescent="0.2">
+      <c r="A57" s="10">
+        <v>14</v>
+      </c>
+      <c r="B57" t="s">
+        <v>8</v>
+      </c>
+      <c r="C57" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="E57" s="4">
+        <v>45607</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated issue log with issue #20 and resolution.
</commit_message>
<xml_diff>
--- a/doc/assurance/ZoneAlertService/4-Issues/issues.xlsx
+++ b/doc/assurance/ZoneAlertService/4-Issues/issues.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Dependable/Contracts/ASTRA/Deliverables/OpenUxAS-ZoneAlert/doc/assurance/ZoneAlertService/4-Issues/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49B6F53B-DB81-FD4E-94C5-DCCB3FB049E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F175771E-4E33-B946-91FA-1FC311A929E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2080" yWindow="500" windowWidth="33760" windowHeight="20740" xr2:uid="{C9A58872-7F3C-C947-8C7B-D579EDD417B1}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="109">
   <si>
     <t>Status</t>
   </si>
@@ -359,6 +359,12 @@
   </si>
   <si>
     <t>Updated the code to be compliant with the architecture. processReceivedLmcpMessage now calls subfunctions as defined in the architecture to handle the logic for the received message types.</t>
+  </si>
+  <si>
+    <t>Copying and passting the code for re-use from RoutePlanningVisbilityService, in order to utilize the same computed geomtry as the route planner, is not future- safe enough to keep Route planning and zone alerting geomertry in sync</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Update the the RoutePlanningVisibilityService to allow SimpleZoneAlertComputer to be a friend, able to access non-public members of the RoutePlanningVisibbilityService. This allows us to carefully use its internal geometry computqtions . We only need the bindPointsforeometry stuff. Modified everything to work this way and got rid of the copied code. </t>
   </si>
 </sst>
 </file>
@@ -799,7 +805,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50891FDD-30FA-7E4F-8B50-3438F693C3DF}">
-  <dimension ref="A1:I71"/>
+  <dimension ref="A1:I72"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.5" style="10" customWidth="1"/>
@@ -1702,6 +1708,9 @@
       <c r="E57" s="4">
         <v>45607</v>
       </c>
+      <c r="F57" s="9">
+        <v>45682</v>
+      </c>
       <c r="G57" s="4">
         <v>45681</v>
       </c>
@@ -1788,6 +1797,12 @@
       <c r="C61" s="6" t="s">
         <v>92</v>
       </c>
+      <c r="E61" s="4">
+        <v>45705</v>
+      </c>
+      <c r="F61" s="9">
+        <v>45706</v>
+      </c>
       <c r="H61" s="6" t="s">
         <v>93</v>
       </c>
@@ -1797,6 +1812,9 @@
     </row>
     <row r="62" spans="1:9" ht="51" x14ac:dyDescent="0.2">
       <c r="F62" s="4"/>
+      <c r="G62" s="4">
+        <v>45705</v>
+      </c>
       <c r="H62" s="6" t="s">
         <v>100</v>
       </c>
@@ -1818,7 +1836,7 @@
         <v>45706</v>
       </c>
       <c r="F63" s="4">
-        <v>45706</v>
+        <v>45707</v>
       </c>
       <c r="G63" s="4">
         <v>45706</v>
@@ -1880,6 +1898,12 @@
       <c r="C69" s="6" t="s">
         <v>102</v>
       </c>
+      <c r="E69" s="4">
+        <v>45707</v>
+      </c>
+      <c r="F69" s="9">
+        <v>45707</v>
+      </c>
       <c r="G69" s="4">
         <v>45707</v>
       </c>
@@ -1914,6 +1938,9 @@
       <c r="E71" s="4">
         <v>45707</v>
       </c>
+      <c r="F71" s="9">
+        <v>45708</v>
+      </c>
       <c r="G71" s="4">
         <v>45708</v>
       </c>
@@ -1921,6 +1948,32 @@
         <v>106</v>
       </c>
       <c r="I71" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="72" spans="1:9" ht="85" x14ac:dyDescent="0.2">
+      <c r="A72" s="10">
+        <v>21</v>
+      </c>
+      <c r="B72" t="s">
+        <v>20</v>
+      </c>
+      <c r="C72" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="E72" s="4">
+        <v>45709</v>
+      </c>
+      <c r="F72" s="9">
+        <v>45709</v>
+      </c>
+      <c r="G72" s="4">
+        <v>45709</v>
+      </c>
+      <c r="H72" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="I72" t="s">
         <v>20</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Updated issues log for recent testing and debugging.
</commit_message>
<xml_diff>
--- a/doc/assurance/ZoneAlertService/4-Issues/issues.xlsx
+++ b/doc/assurance/ZoneAlertService/4-Issues/issues.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Dependable/Contracts/ASTRA/Deliverables/OpenUxAS-ZoneAlert/doc/assurance/ZoneAlertService/4-Issues/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11A823DD-B9A4-1945-8432-3726FB5BCB49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BA400A7-C56F-2645-AC3D-B4632B361F50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2080" yWindow="500" windowWidth="33760" windowHeight="20740" xr2:uid="{C9A58872-7F3C-C947-8C7B-D579EDD417B1}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="157">
   <si>
     <t>Status</t>
   </si>
@@ -407,6 +407,108 @@
   </si>
   <si>
     <t>HL-1-1-2-1 and HL-1-1-2-2 are split up in their assurance within the correctness argument across multiple aspect branches</t>
+  </si>
+  <si>
+    <t>Processed zones all have zero id</t>
+  </si>
+  <si>
+    <t>Fixed code that should have set merged zone ids. Fixed zone type assignment as well</t>
+  </si>
+  <si>
+    <t>Tests now pass showing correct id numbering and zone type assignment</t>
+  </si>
+  <si>
+    <t>Computation of endposition tranposes x and y coordinates</t>
+  </si>
+  <si>
+    <t>Code examined and repaired by inspection</t>
+  </si>
+  <si>
+    <t>Tests show desired behavior</t>
+  </si>
+  <si>
+    <t>No means of resetting coordinate conversion between unit / compositional tests in gtest</t>
+  </si>
+  <si>
+    <t>Added Reset static function to CUnitConversions class to enable reset of starting reference for flat plane tangent to earth</t>
+  </si>
+  <si>
+    <t>computeViolations is building the start position of a vehicle using Cposition, which assumes lat and long in radians. We must first convert from degrees to radians.</t>
+  </si>
+  <si>
+    <t>Added code to correctly generate the starting position with knowledge that reported position is in lat, long, altitude in degrees and meters, and Cposition must have that converted to radians first. Tracing shows correct function. (Would ormally add a test at unit level here but no time)</t>
+  </si>
+  <si>
+    <t>Validation Question: Would the user prefer the location of violations in east, north, alt of the tangent plane (and relative to merged zone coords) or in the original latituce, longitude, altitude, or both?</t>
+  </si>
+  <si>
+    <t>Failed check for closest intersection in SimpleZoneAlertComputer::findClosestIntersection. It accepts the last intersection it checks</t>
+  </si>
+  <si>
+    <t>Examining code shows that it is using some 'farthest' calculation when it should be looking for the 'closest'. Failed record closest interation. Simple error</t>
+  </si>
+  <si>
+    <t>Corrected code to perform correct closest check</t>
+  </si>
+  <si>
+    <t>Tests pass checking that the closst intersection function works correctly</t>
+  </si>
+  <si>
+    <t>Validation Question: Polygon intersection function appears to have limited accuracy (0.5 meters) for a horizontal intercept detection. Is this acceptable?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tracing in functions shows some kind of rounding performed that may impact results </t>
+  </si>
+  <si>
+    <t>Time to intercept is promoting TO INTEGER somewhere during computation of imminent violations</t>
+  </si>
+  <si>
+    <t>Confirmed the time to intercept of a test example is declared as 1 when it should be 1.56</t>
+  </si>
+  <si>
+    <t>Found all functions assuming int64 time in milliseconds. Copnverted messages and all functions to use double-valued time in seconds</t>
+  </si>
+  <si>
+    <t>Converted code for reported time to be future time in seconds ahead of vehicle state report, rather than clock time</t>
+  </si>
+  <si>
+    <t>Tests show time is correctly reported</t>
+  </si>
+  <si>
+    <t>Vertices in boundary sets for ZoneAlertComputer contain incorrect indexes. They need to restart at zero</t>
+  </si>
+  <si>
+    <t>Confirmed that the indexes stored for the boundary of the second processed zone are incorrect index numbers that need to be reset to match those stored with vertices.</t>
+  </si>
+  <si>
+    <t>OK, so the problem is that the polygon, when taking parameters of x and y directly, associates X with North and Y with East</t>
+  </si>
+  <si>
+    <t>Beyond the first merged zones, remaining zones are not detecting intersections of vehicle trajectory with their zone boundaries.</t>
+  </si>
+  <si>
+    <t>Failure reproduced with indiation that Polygon vertex indeces and boundary vertex positions are correct, but failure is occuring in Polgon::findINtersections function.</t>
+  </si>
+  <si>
+    <t>Interactive debugging inspection of Polygon shows that the edgesArray stores records of the two vertex indecises for each edge, which are still set to the vertex indeces from the original merged polygons, which assume that global array of positions which we don't use. Hence we will need to modify our merge code to update edge vertex indices ith the correct edge vertex indeces.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fixed indeces for edges on non-first merged zone during zone merge results recording. Tests passed </t>
+  </si>
+  <si>
+    <t>Arbitrary, non-deterministic memory corruption (incorrect memory usage by source code) producing sometimes random values in violation-&gt;getInterceptPosition()-&gt;getNorth()</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reproduced. Error is incorrect passing of address of local stack vector element as return value. </t>
+  </si>
+  <si>
+    <t>Fixed by creating a copy of the relevant CPOsition as new object to return. Testing shows success.</t>
+  </si>
+  <si>
+    <t>Returned violation reported time to future absolute time in milliseconds so that it is not relative to decoupled reported state times</t>
+  </si>
+  <si>
+    <t>Relative violation in future time is not useful if the receiver doesn't know what the vehicle state report times were.</t>
   </si>
 </sst>
 </file>
@@ -491,7 +593,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
@@ -508,14 +610,10 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -533,6 +631,13 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -847,10 +952,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50891FDD-30FA-7E4F-8B50-3438F693C3DF}">
-  <dimension ref="A1:I83"/>
+  <dimension ref="A1:I106"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14.5" style="10" customWidth="1"/>
+    <col min="1" max="1" width="14.5" style="19" customWidth="1"/>
     <col min="2" max="2" width="13.6640625" customWidth="1"/>
     <col min="3" max="4" width="47.5" style="6" customWidth="1"/>
     <col min="5" max="5" width="15.1640625" style="4" customWidth="1"/>
@@ -861,22 +966,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="17" t="s">
         <v>2</v>
       </c>
       <c r="B1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="15" t="s">
+      <c r="C1" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="D1" s="15" t="s">
+      <c r="D1" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="E1" s="16" t="s">
+      <c r="E1" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="F1" s="17" t="s">
+      <c r="F1" s="15" t="s">
         <v>7</v>
       </c>
       <c r="G1" s="11" t="s">
@@ -886,12 +991,12 @@
       <c r="I1" s="11"/>
     </row>
     <row r="2" spans="1:9" ht="18" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="13"/>
-      <c r="B2" s="14"/>
-      <c r="C2" s="15"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="17"/>
+      <c r="A2" s="18"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="15"/>
       <c r="G2" s="2" t="s">
         <v>5</v>
       </c>
@@ -903,7 +1008,7 @@
       </c>
     </row>
     <row r="3" spans="1:9" ht="51" x14ac:dyDescent="0.2">
-      <c r="A3" s="10">
+      <c r="A3" s="19">
         <v>1</v>
       </c>
       <c r="B3" t="s">
@@ -1017,7 +1122,7 @@
       </c>
     </row>
     <row r="12" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A12" s="10">
+      <c r="A12" s="19">
         <v>2</v>
       </c>
       <c r="B12" t="s">
@@ -1065,7 +1170,7 @@
       </c>
     </row>
     <row r="15" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A15" s="10">
+      <c r="A15" s="19">
         <v>3</v>
       </c>
       <c r="B15" t="s">
@@ -1105,7 +1210,7 @@
       </c>
     </row>
     <row r="17" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A17" s="10">
+      <c r="A17" s="19">
         <v>4</v>
       </c>
       <c r="B17" t="s">
@@ -1145,7 +1250,7 @@
       </c>
     </row>
     <row r="19" spans="1:9" ht="272" x14ac:dyDescent="0.2">
-      <c r="A19" s="10">
+      <c r="A19" s="19">
         <v>1.1000000000000001</v>
       </c>
       <c r="B19" t="s">
@@ -1182,7 +1287,7 @@
       </c>
     </row>
     <row r="21" spans="1:9" ht="51" x14ac:dyDescent="0.2">
-      <c r="A21" s="10">
+      <c r="A21" s="19">
         <v>1.2</v>
       </c>
       <c r="B21" t="s">
@@ -1219,7 +1324,7 @@
       </c>
     </row>
     <row r="23" spans="1:9" ht="68" x14ac:dyDescent="0.2">
-      <c r="A23" s="10">
+      <c r="A23" s="19">
         <v>5</v>
       </c>
       <c r="B23" t="s">
@@ -1256,7 +1361,7 @@
       </c>
     </row>
     <row r="25" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A25" s="10">
+      <c r="A25" s="19">
         <v>1.3</v>
       </c>
       <c r="B25" t="s">
@@ -1282,7 +1387,7 @@
       </c>
     </row>
     <row r="26" spans="1:9" ht="51" x14ac:dyDescent="0.2">
-      <c r="A26" s="10">
+      <c r="A26" s="19">
         <v>1.4</v>
       </c>
       <c r="B26" t="s">
@@ -1308,7 +1413,7 @@
       </c>
     </row>
     <row r="27" spans="1:9" ht="187" x14ac:dyDescent="0.2">
-      <c r="A27" s="10">
+      <c r="A27" s="19">
         <v>6</v>
       </c>
       <c r="B27" t="s">
@@ -1334,7 +1439,7 @@
       </c>
     </row>
     <row r="28" spans="1:9" ht="68" x14ac:dyDescent="0.2">
-      <c r="A28" s="10">
+      <c r="A28" s="19">
         <v>7</v>
       </c>
       <c r="B28" t="s">
@@ -1360,7 +1465,7 @@
       </c>
     </row>
     <row r="29" spans="1:9" ht="119" x14ac:dyDescent="0.2">
-      <c r="A29" s="10">
+      <c r="A29" s="19">
         <v>8</v>
       </c>
       <c r="B29" t="s">
@@ -1430,7 +1535,7 @@
       </c>
     </row>
     <row r="34" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A34" s="10">
+      <c r="A34" s="19">
         <v>9</v>
       </c>
       <c r="B34" t="s">
@@ -1456,7 +1561,7 @@
       </c>
     </row>
     <row r="35" spans="1:9" ht="68" x14ac:dyDescent="0.2">
-      <c r="A35" s="10">
+      <c r="A35" s="19">
         <v>10</v>
       </c>
       <c r="B35" t="s">
@@ -1479,7 +1584,7 @@
       </c>
     </row>
     <row r="36" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A36" s="10">
+      <c r="A36" s="19">
         <v>11</v>
       </c>
       <c r="B36" t="s">
@@ -1510,7 +1615,7 @@
       </c>
     </row>
     <row r="38" spans="1:9" ht="68" x14ac:dyDescent="0.2">
-      <c r="A38" s="10">
+      <c r="A38" s="19">
         <v>12</v>
       </c>
       <c r="B38" t="s">
@@ -1555,7 +1660,7 @@
       </c>
     </row>
     <row r="41" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A41" s="10" t="s">
+      <c r="A41" s="19" t="s">
         <v>76</v>
       </c>
       <c r="G41" s="4">
@@ -1668,7 +1773,7 @@
       </c>
     </row>
     <row r="52" spans="1:9" ht="102" x14ac:dyDescent="0.2">
-      <c r="A52" s="10">
+      <c r="A52" s="19">
         <v>13</v>
       </c>
       <c r="B52" t="s">
@@ -1738,7 +1843,7 @@
       </c>
     </row>
     <row r="57" spans="1:9" ht="68" x14ac:dyDescent="0.2">
-      <c r="A57" s="10">
+      <c r="A57" s="19">
         <v>14</v>
       </c>
       <c r="B57" t="s">
@@ -1764,7 +1869,7 @@
       </c>
     </row>
     <row r="58" spans="1:9" ht="51" x14ac:dyDescent="0.2">
-      <c r="A58" s="10">
+      <c r="A58" s="19">
         <v>15</v>
       </c>
       <c r="B58" t="s">
@@ -1790,7 +1895,7 @@
       </c>
     </row>
     <row r="59" spans="1:9" ht="85" x14ac:dyDescent="0.2">
-      <c r="A59" s="10">
+      <c r="A59" s="19">
         <v>16</v>
       </c>
       <c r="B59" t="s">
@@ -1830,7 +1935,7 @@
       </c>
     </row>
     <row r="61" spans="1:9" ht="85" x14ac:dyDescent="0.2">
-      <c r="A61" s="10">
+      <c r="A61" s="19">
         <v>17</v>
       </c>
       <c r="B61" t="s">
@@ -1865,7 +1970,7 @@
       </c>
     </row>
     <row r="63" spans="1:9" ht="51" x14ac:dyDescent="0.2">
-      <c r="A63" s="10">
+      <c r="A63" s="19">
         <v>18</v>
       </c>
       <c r="B63" t="s">
@@ -1931,7 +2036,7 @@
       </c>
     </row>
     <row r="69" spans="1:9" ht="85" x14ac:dyDescent="0.2">
-      <c r="A69" s="10">
+      <c r="A69" s="19">
         <v>19</v>
       </c>
       <c r="B69" t="s">
@@ -1968,7 +2073,7 @@
       </c>
     </row>
     <row r="71" spans="1:9" ht="136" x14ac:dyDescent="0.2">
-      <c r="A71" s="10">
+      <c r="A71" s="19">
         <v>20</v>
       </c>
       <c r="B71" t="s">
@@ -1994,7 +2099,7 @@
       </c>
     </row>
     <row r="72" spans="1:9" ht="85" x14ac:dyDescent="0.2">
-      <c r="A72" s="10">
+      <c r="A72" s="19">
         <v>21</v>
       </c>
       <c r="B72" t="s">
@@ -2020,7 +2125,7 @@
       </c>
     </row>
     <row r="73" spans="1:9" ht="102" x14ac:dyDescent="0.2">
-      <c r="A73" s="10">
+      <c r="A73" s="19">
         <v>22</v>
       </c>
       <c r="B73" t="s">
@@ -2034,7 +2139,7 @@
       </c>
     </row>
     <row r="74" spans="1:9" ht="119" x14ac:dyDescent="0.2">
-      <c r="A74" s="10">
+      <c r="A74" s="19">
         <v>23</v>
       </c>
       <c r="B74" t="s">
@@ -2048,7 +2153,7 @@
       </c>
     </row>
     <row r="75" spans="1:9" ht="51" x14ac:dyDescent="0.2">
-      <c r="A75" s="10">
+      <c r="A75" s="19">
         <v>24</v>
       </c>
       <c r="B75" t="s">
@@ -2062,7 +2167,7 @@
       </c>
     </row>
     <row r="76" spans="1:9" ht="85" x14ac:dyDescent="0.2">
-      <c r="A76" s="10">
+      <c r="A76" s="19">
         <v>25</v>
       </c>
       <c r="B76" t="s">
@@ -2076,7 +2181,7 @@
       </c>
     </row>
     <row r="77" spans="1:9" ht="68" x14ac:dyDescent="0.2">
-      <c r="A77" s="10">
+      <c r="A77" s="19">
         <v>26</v>
       </c>
       <c r="B77" t="s">
@@ -2090,7 +2195,7 @@
       </c>
     </row>
     <row r="78" spans="1:9" ht="68" x14ac:dyDescent="0.2">
-      <c r="A78" s="10">
+      <c r="A78" s="19">
         <v>27</v>
       </c>
       <c r="B78" t="s">
@@ -2104,7 +2209,7 @@
       </c>
     </row>
     <row r="79" spans="1:9" ht="102" x14ac:dyDescent="0.2">
-      <c r="A79" s="10">
+      <c r="A79" s="19">
         <v>28</v>
       </c>
       <c r="B79" t="s">
@@ -2118,7 +2223,7 @@
       </c>
     </row>
     <row r="80" spans="1:9" ht="68" x14ac:dyDescent="0.2">
-      <c r="A80" s="10">
+      <c r="A80" s="19">
         <v>29</v>
       </c>
       <c r="B80" t="s">
@@ -2141,7 +2246,7 @@
       </c>
     </row>
     <row r="81" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A81" s="10">
+      <c r="A81" s="19">
         <v>30</v>
       </c>
       <c r="B81" t="s">
@@ -2164,7 +2269,7 @@
       </c>
     </row>
     <row r="82" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A82" s="10">
+      <c r="A82" s="19">
         <v>31</v>
       </c>
       <c r="B82" t="s">
@@ -2187,7 +2292,7 @@
       </c>
     </row>
     <row r="83" spans="1:9" ht="51" x14ac:dyDescent="0.2">
-      <c r="A83" s="10">
+      <c r="A83" s="19">
         <v>32</v>
       </c>
       <c r="B83" t="s">
@@ -2198,6 +2303,430 @@
       </c>
       <c r="E83" s="4">
         <v>45730</v>
+      </c>
+    </row>
+    <row r="84" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A84" s="19">
+        <v>33</v>
+      </c>
+      <c r="B84" t="s">
+        <v>20</v>
+      </c>
+      <c r="C84" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="E84" s="4">
+        <v>45747</v>
+      </c>
+      <c r="F84" s="9">
+        <v>45747</v>
+      </c>
+      <c r="G84" s="4">
+        <v>45747</v>
+      </c>
+      <c r="H84" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="I84" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="85" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="G85" s="4">
+        <v>45747</v>
+      </c>
+      <c r="H85" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="I85" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="86" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="A86" s="19">
+        <v>34</v>
+      </c>
+      <c r="B86" t="s">
+        <v>20</v>
+      </c>
+      <c r="C86" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="E86" s="4">
+        <v>45747</v>
+      </c>
+      <c r="F86" s="9">
+        <v>45747</v>
+      </c>
+      <c r="G86" s="9">
+        <v>45747</v>
+      </c>
+      <c r="H86" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I86" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="87" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="G87" s="9">
+        <v>45747</v>
+      </c>
+      <c r="H87" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="I87" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="88" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="A88" s="19">
+        <v>35</v>
+      </c>
+      <c r="B88" t="s">
+        <v>20</v>
+      </c>
+      <c r="C88" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="E88" s="4">
+        <v>45748</v>
+      </c>
+      <c r="F88" s="9">
+        <v>45748</v>
+      </c>
+      <c r="G88" s="4">
+        <v>45748</v>
+      </c>
+      <c r="H88" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="I88" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="89" spans="1:9" ht="68" x14ac:dyDescent="0.2">
+      <c r="A89" s="19">
+        <v>36</v>
+      </c>
+      <c r="B89" t="s">
+        <v>20</v>
+      </c>
+      <c r="C89" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="E89" s="4">
+        <v>45748</v>
+      </c>
+      <c r="F89" s="9">
+        <v>45748</v>
+      </c>
+      <c r="G89" s="4">
+        <v>45748</v>
+      </c>
+      <c r="H89" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="I89" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="90" spans="1:9" ht="68" x14ac:dyDescent="0.2">
+      <c r="A90" s="19">
+        <v>37</v>
+      </c>
+      <c r="B90" t="s">
+        <v>8</v>
+      </c>
+      <c r="C90" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="E90" s="4">
+        <v>45748</v>
+      </c>
+      <c r="F90" s="9">
+        <v>45748</v>
+      </c>
+    </row>
+    <row r="91" spans="1:9" ht="51" x14ac:dyDescent="0.2">
+      <c r="A91" s="19">
+        <v>38</v>
+      </c>
+      <c r="B91" t="s">
+        <v>20</v>
+      </c>
+      <c r="C91" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="E91" s="4">
+        <v>45748</v>
+      </c>
+      <c r="F91" s="9">
+        <v>45748</v>
+      </c>
+      <c r="G91" s="4">
+        <v>45748</v>
+      </c>
+      <c r="H91" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="I91" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="92" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="G92" s="4">
+        <v>45748</v>
+      </c>
+      <c r="H92" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="I92" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="93" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="G93" s="4">
+        <v>45748</v>
+      </c>
+      <c r="H93" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="I93" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="94" spans="1:9" ht="51" x14ac:dyDescent="0.2">
+      <c r="A94" s="19">
+        <v>39</v>
+      </c>
+      <c r="B94" t="s">
+        <v>8</v>
+      </c>
+      <c r="C94" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="E94" s="4">
+        <v>45748</v>
+      </c>
+      <c r="F94" s="9">
+        <v>45748</v>
+      </c>
+      <c r="G94" s="4">
+        <v>45748</v>
+      </c>
+      <c r="H94" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="I94" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="95" spans="1:9" ht="55" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A95" s="19">
+        <v>40</v>
+      </c>
+      <c r="B95" t="s">
+        <v>20</v>
+      </c>
+      <c r="C95" s="10" t="s">
+        <v>140</v>
+      </c>
+      <c r="E95" s="4">
+        <v>45748</v>
+      </c>
+      <c r="F95" s="9">
+        <v>45748</v>
+      </c>
+      <c r="G95" s="4">
+        <v>45748</v>
+      </c>
+      <c r="H95" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="I95" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="96" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="G96" s="4">
+        <v>45748</v>
+      </c>
+      <c r="H96" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="I96" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="97" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="G97" s="4">
+        <v>45748</v>
+      </c>
+      <c r="H97" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="I97" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="98" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="G98" s="4">
+        <v>45748</v>
+      </c>
+      <c r="H98" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="I98" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="99" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="A99" s="19">
+        <v>41</v>
+      </c>
+      <c r="B99" t="s">
+        <v>20</v>
+      </c>
+      <c r="C99" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="E99" s="4">
+        <v>45748</v>
+      </c>
+      <c r="F99" s="9">
+        <v>45748</v>
+      </c>
+      <c r="G99" s="4">
+        <v>45748</v>
+      </c>
+      <c r="H99" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="I99" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="100" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="G100" s="4">
+        <v>45748</v>
+      </c>
+      <c r="H100" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="I100" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="101" spans="1:9" ht="51" x14ac:dyDescent="0.2">
+      <c r="A101" s="19">
+        <v>42</v>
+      </c>
+      <c r="B101" t="s">
+        <v>20</v>
+      </c>
+      <c r="C101" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="E101" s="4">
+        <v>45748</v>
+      </c>
+      <c r="F101" s="9">
+        <v>45749</v>
+      </c>
+      <c r="G101" s="4">
+        <v>45748</v>
+      </c>
+      <c r="H101" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="I101" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="102" spans="1:9" ht="85" x14ac:dyDescent="0.2">
+      <c r="G102" s="4">
+        <v>45749</v>
+      </c>
+      <c r="H102" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="I102" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="103" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="G103" s="4">
+        <v>45749</v>
+      </c>
+      <c r="H103" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="I103" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="104" spans="1:9" ht="68" x14ac:dyDescent="0.2">
+      <c r="A104" s="19">
+        <v>43</v>
+      </c>
+      <c r="B104" t="s">
+        <v>20</v>
+      </c>
+      <c r="C104" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="E104" s="4">
+        <v>45749</v>
+      </c>
+      <c r="F104" s="9">
+        <v>45749</v>
+      </c>
+      <c r="G104" s="4">
+        <v>45749</v>
+      </c>
+      <c r="H104" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="I104" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="105" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="G105" s="4">
+        <v>45749</v>
+      </c>
+      <c r="H105" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="I105" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="106" spans="1:9" ht="51" x14ac:dyDescent="0.2">
+      <c r="A106" s="19">
+        <v>44</v>
+      </c>
+      <c r="B106" t="s">
+        <v>20</v>
+      </c>
+      <c r="C106" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="E106" s="4">
+        <v>45749</v>
+      </c>
+      <c r="F106" s="9">
+        <v>45749</v>
+      </c>
+      <c r="G106" s="4">
+        <v>45749</v>
+      </c>
+      <c r="H106" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="I106" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Issues from operation of first service demo.
</commit_message>
<xml_diff>
--- a/doc/assurance/ZoneAlertService/4-Issues/issues.xlsx
+++ b/doc/assurance/ZoneAlertService/4-Issues/issues.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Dependable/Contracts/ASTRA/Deliverables/OpenUxAS-ZoneAlert/doc/assurance/ZoneAlertService/4-Issues/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BA400A7-C56F-2645-AC3D-B4632B361F50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF6E8B88-4A4D-524B-B36F-8A13806FB3D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2080" yWindow="500" windowWidth="33760" windowHeight="20740" xr2:uid="{C9A58872-7F3C-C947-8C7B-D579EDD417B1}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="169">
   <si>
     <t>Status</t>
   </si>
@@ -509,6 +509,42 @@
   </si>
   <si>
     <t>Relative violation in future time is not useful if the receiver doesn't know what the vehicle state report times were.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scenarios will often declare vehicle states before declaring automations, making automations the wrong message to trigger Zone Merging, as by the time that message goes out, vehicles have already reported state, checked if they have a keep in zone, found no zones to check, and therefore have no keep-in zone. </t>
+  </si>
+  <si>
+    <t>We could change the logic of keep-in zone assignment to be that a vehicle belongs to any keep-in zone it enters. But we have to validate that requirement with Stakeholders. In addition, the automation request is definitely not good enough. Another option is to always have the last state reported position of a vehicle be recorded and 'capture' any vehicles in any newly declared merged keep-in zones.  So two questions: When to trigger merging and semantics for keep-in zone owners of a vehicle.</t>
+  </si>
+  <si>
+    <t>Decided to change semantics so that a vehicle without a keep-in zone will become attached to the first keep-in zone it enters, if ever</t>
+  </si>
+  <si>
+    <t>Tested and works, added test specifically for this condition to the tests generated</t>
+  </si>
+  <si>
+    <t>Added a new validation check issue #46</t>
+  </si>
+  <si>
+    <t>Is it acceptable semantics for vehicles to belong to the first keep-in zone they happen to be in or wander into?</t>
+  </si>
+  <si>
+    <t>Demos confirm that keep out zone imminent violation time spikes just before the vehicle enters the keep-out zone. And it enters close to the predicted time. Hypothesis: When near boundary, there is an innacuracy in time computation. Furthermore, this may be due to loss of precision. Will require investigation.</t>
+  </si>
+  <si>
+    <t>Ask stakeholders if the first time a vehicle wanders into a keep-in zone, it belongs to that zone, is an acceptible semantic. If so, update requirements. Otherwise, reo-open issue #45 and find another solution to that issue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calculation of time of initial keep out zone imminent violtions seems to experience a jump/spike near the boundary and becomes temporarily inaccurate </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calculation of time of second keep-out zone imminent violations appears to be off by about 300 milliseconds from actual violation time starting. </t>
+  </si>
+  <si>
+    <t>Hypothesis: We might be only updating vehicle states roughly once every 300-500 milliseconds, which would be why the time of traversal and first report of active violation wouldn't be the same.</t>
+  </si>
+  <si>
+    <t>Checking timestamps of reports, this apepars to be the case. Closing.</t>
   </si>
 </sst>
 </file>
@@ -952,7 +988,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50891FDD-30FA-7E4F-8B50-3438F693C3DF}">
-  <dimension ref="A1:I106"/>
+  <dimension ref="A1:I114"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.5" style="19" customWidth="1"/>
@@ -2726,6 +2762,136 @@
         <v>155</v>
       </c>
       <c r="I106" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="107" spans="1:9" ht="102" x14ac:dyDescent="0.2">
+      <c r="A107" s="19">
+        <v>45</v>
+      </c>
+      <c r="B107" t="s">
+        <v>20</v>
+      </c>
+      <c r="C107" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="E107" s="4">
+        <v>45751</v>
+      </c>
+      <c r="G107" s="4">
+        <v>45751</v>
+      </c>
+      <c r="H107" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="I107" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="108" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="G108" s="4">
+        <v>45751</v>
+      </c>
+      <c r="H108" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="I108" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="109" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="G109" s="4">
+        <v>45751</v>
+      </c>
+      <c r="H109" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="I109" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="110" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="G110" s="4">
+        <v>45751</v>
+      </c>
+      <c r="H110" s="6" t="s">
+        <v>161</v>
+      </c>
+      <c r="I110" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="111" spans="1:9" ht="51" x14ac:dyDescent="0.2">
+      <c r="A111" s="19">
+        <v>46</v>
+      </c>
+      <c r="B111" t="s">
+        <v>8</v>
+      </c>
+      <c r="C111" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="E111" s="4">
+        <v>45751</v>
+      </c>
+      <c r="H111" s="6" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="112" spans="1:9" ht="68" x14ac:dyDescent="0.2">
+      <c r="A112" s="19">
+        <v>47</v>
+      </c>
+      <c r="B112" t="s">
+        <v>8</v>
+      </c>
+      <c r="C112" s="6" t="s">
+        <v>165</v>
+      </c>
+      <c r="E112" s="4">
+        <v>45751</v>
+      </c>
+      <c r="H112" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="I112" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="113" spans="1:9" ht="51" x14ac:dyDescent="0.2">
+      <c r="A113" s="19">
+        <v>48</v>
+      </c>
+      <c r="B113" t="s">
+        <v>8</v>
+      </c>
+      <c r="C113" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="E113" s="4">
+        <v>45751</v>
+      </c>
+      <c r="F113" s="9">
+        <v>45751</v>
+      </c>
+      <c r="G113" s="4">
+        <v>45751</v>
+      </c>
+      <c r="H113" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="I113" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="114" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="G114" s="4">
+        <v>45751</v>
+      </c>
+      <c r="H114" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="I114" t="s">
         <v>20</v>
       </c>
     </row>

</xml_diff>